<commit_message>
FHIR-56242: Rename MembersToMatch to MemberBundle in Provider Member Match
- Rename MembersToMatch parameter to MemberBundle in OperationDefinition,
  Parameters profile, and examples to align with BulkMemberMatch naming
- Rename TreatmentAttestation parameter to Consent
- Fix ProviderConsent references back to ProviderTreatmentAttestation
  (profile was not renamed)
- Fix redundant documentation string in Operation-provider-member-match
- Add FHIR-56242 to STU 2.2.0 change history table
- Update fsh-generated and output artifacts

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/StructureDefinition-provider-parameters-multi-member-match-bundle-in.xlsx
+++ b/output/StructureDefinition-provider-parameters-multi-member-match-bundle-in.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-19T09:51:30-04:00</t>
+    <t>2026-03-31T21:00:10-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -513,10 +513,10 @@
     <t>Only one level of nested parameters is allowed.</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch</t>
-  </si>
-  <si>
-    <t>MembersToMatch</t>
+    <t>Parameters.parameter:MemberBundle</t>
+  </si>
+  <si>
+    <t>MemberBundle</t>
   </si>
   <si>
     <t>Operation Parameter</t>
@@ -525,16 +525,16 @@
     <t>A parameter passed to or received from the operation.</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.id</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.extension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.modifierExtension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.name</t>
+    <t>Parameters.parameter:MemberBundle.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.name</t>
   </si>
   <si>
     <t>Member elements to match for provider access</t>
@@ -543,13 +543,13 @@
     <t>A repeating parameter containing current member demographics, current coverage information, and provider treatment attestation for a single member. The name aligns with the ProviderMemberMatch OperationDefinition.</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.value[x]</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.resource</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part</t>
+    <t>Parameters.parameter:MemberBundle.value[x]</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.resource</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part</t>
   </si>
   <si>
     <t>3</t>
@@ -561,64 +561,64 @@
     <t>The individual components required for a provider to request access to member data: current patient demographics, current coverage, and provider treatment attestation.</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part.id</t>
+    <t>Parameters.parameter:MemberBundle.part.id</t>
   </si>
   <si>
     <t>Parameters.parameter.part.id</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part.extension</t>
+    <t>Parameters.parameter:MemberBundle.part.extension</t>
   </si>
   <si>
     <t>Parameters.parameter.part.extension</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part.modifierExtension</t>
+    <t>Parameters.parameter:MemberBundle.part.modifierExtension</t>
   </si>
   <si>
     <t>Parameters.parameter.part.modifierExtension</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part.name</t>
+    <t>Parameters.parameter:MemberBundle.part.name</t>
   </si>
   <si>
     <t>Parameters.parameter.part.name</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part.value[x]</t>
+    <t>Parameters.parameter:MemberBundle.part.value[x]</t>
   </si>
   <si>
     <t>Parameters.parameter.part.value[x]</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part.resource</t>
+    <t>Parameters.parameter:MemberBundle.part.resource</t>
   </si>
   <si>
     <t>Parameters.parameter.part.resource</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part.part</t>
+    <t>Parameters.parameter:MemberBundle.part.part</t>
   </si>
   <si>
     <t>Parameters.parameter.part.part</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient</t>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient</t>
   </si>
   <si>
     <t>MemberPatient</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient.id</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient.extension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient.modifierExtension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient.name</t>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient.name</t>
   </si>
   <si>
     <t>Current member demographics</t>
@@ -627,10 +627,10 @@
     <t>Current patient demographic information as known by the provider (from provider's EMR or patient-provided information).</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient.value[x]</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient.resource</t>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient.value[x]</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient.resource</t>
   </si>
   <si>
     <t xml:space="preserve">SubjectOfCare Client Resident
@@ -650,25 +650,25 @@
     <t>Patient[classCode=PAT]</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:MemberPatient.part</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch</t>
+    <t>Parameters.parameter:MemberBundle.part:MemberPatient.part</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch</t>
   </si>
   <si>
     <t>CoverageToMatch</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch.id</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch.extension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch.modifierExtension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch.name</t>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch.name</t>
   </si>
   <si>
     <t>Current member coverage</t>
@@ -677,10 +677,10 @@
     <t>The member's current active coverage with the payer (typically from insurance card or eligibility verification).</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch.value[x]</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch.resource</t>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch.value[x]</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch.resource</t>
   </si>
   <si>
     <t xml:space="preserve">Coverage {http://hl7.org/fhir/us/davinci-hrex/StructureDefinition/hrex-coverage}
@@ -699,25 +699,25 @@
     <t>Coverage</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToMatch.part</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation</t>
-  </si>
-  <si>
-    <t>TreatmentAttestation</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation.id</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation.extension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation.modifierExtension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation.name</t>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToMatch.part</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:Consent</t>
+  </si>
+  <si>
+    <t>Consent</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:Consent.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:Consent.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:Consent.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:Consent.name</t>
   </si>
   <si>
     <t>Provider treatment attestation</t>
@@ -726,10 +726,10 @@
     <t>Provider's attestation of an active treatment relationship with the member. This is NOT patient consent for payer-to-payer data exchange, but rather the provider's certification that they have a treatment relationship justifying access to the member's data.</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation.value[x]</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation.resource</t>
+    <t>Parameters.parameter:MemberBundle.part:Consent.value[x]</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:Consent.resource</t>
   </si>
   <si>
     <t xml:space="preserve">Consent {http://hl7.org/fhir/us/davinci-pdex/StructureDefinition/provider-treatment-relationship-consent}
@@ -751,25 +751,25 @@
     <t>FinancialConsent</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:TreatmentAttestation.part</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink</t>
+    <t>Parameters.parameter:MemberBundle.part:Consent.part</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink</t>
   </si>
   <si>
     <t>CoverageToLink</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink.id</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink.extension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink.modifierExtension</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink.name</t>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink.id</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink.extension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink.modifierExtension</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink.name</t>
   </si>
   <si>
     <t>Optional coverage to link (typically not used)</t>
@@ -778,10 +778,10 @@
     <t>CoverageToLink is typically not used in provider-initiated member match requests as providers are not linking historical coverage to new coverage. This element is only relevant for payer-to-payer member match operations.</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink.value[x]</t>
-  </si>
-  <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink.resource</t>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink.value[x]</t>
+  </si>
+  <si>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink.resource</t>
   </si>
   <si>
     <t>Insurance or medical plan or a payment agreement</t>
@@ -790,7 +790,7 @@
     <t>This is the Coverage profile which is used to provide insurance information for scheduling an appointment and/or registering a patient.</t>
   </si>
   <si>
-    <t>Parameters.parameter:MembersToMatch.part:CoverageToLink.part</t>
+    <t>Parameters.parameter:MemberBundle.part:CoverageToLink.part</t>
   </si>
 </sst>
 </file>
@@ -1115,9 +1115,9 @@
   <dimension ref="A1:AL61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="66.8828125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="62.0859375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="35.890625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="17.25" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="14.64453125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="23.85546875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.30078125" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="3.953125" customWidth="true" bestFit="true"/>

</xml_diff>